<commit_message>
corrected errors in PNY secure erase figures
</commit_message>
<xml_diff>
--- a/Full final results.xlsx
+++ b/Full final results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\Uni\Dissertation\MScProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0BDB76E-BF8E-4810-8E56-9F0FC9FEA9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C4BBFC-30CF-4971-B200-65B4D61A74C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2085" windowWidth="29040" windowHeight="16440" xr2:uid="{A71FE66F-C5AB-4BD0-A1DF-C1EC892D38EE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A71FE66F-C5AB-4BD0-A1DF-C1EC892D38EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="11" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="61">
   <si>
     <t>Volume</t>
   </si>
@@ -123,21 +123,12 @@
     <t>(114 + 87 + 45) = 246 / 3 = 82 %</t>
   </si>
   <si>
-    <t>(87 / 8,739) = 0.01 * 100 = 1%</t>
-  </si>
-  <si>
-    <t>File Integrity (%) = 1%</t>
-  </si>
-  <si>
     <t>(988 / 8,739) = 0.11 * 100 = 11%</t>
   </si>
   <si>
     <t>Functionality (%) = 11%</t>
   </si>
   <si>
-    <t>(100 + 1 + 11) = 112 / 3 = 37.3 %</t>
-  </si>
-  <si>
     <t>(8,738 / 8,739) = 0.9998 * 100 = 99.98%</t>
   </si>
   <si>
@@ -175,6 +166,57 @@
   </si>
   <si>
     <t>Individual SSD Scenario Average Scores</t>
+  </si>
+  <si>
+    <t>(984 / 8,739) = 0.11 * 100 = 11%</t>
+  </si>
+  <si>
+    <t>File Integrity (%) = 11%</t>
+  </si>
+  <si>
+    <t>(100 + 11 + 11) = 122 / 3 = 40.67 %</t>
+  </si>
+  <si>
+    <t>Autopsy</t>
+  </si>
+  <si>
+    <t>PhotoRec</t>
+  </si>
+  <si>
+    <t>(1,119 / 8,739) = 0.13 * 100 = 13%</t>
+  </si>
+  <si>
+    <t>Volume recovered (%) = 13%</t>
+  </si>
+  <si>
+    <t>File Integrity (%) = 88%</t>
+  </si>
+  <si>
+    <t>(1,119 / 1,119) = 1 * 100 = 100%</t>
+  </si>
+  <si>
+    <t>(13 + 88 + 100) = 201 / 3 = 67 %</t>
+  </si>
+  <si>
+    <t>(983 / 1,119) = 0.88 * 100 = 88%</t>
+  </si>
+  <si>
+    <t>DiskDrill</t>
+  </si>
+  <si>
+    <t>(9,741 / 8,739) = 1.11 * 100 = 110%</t>
+  </si>
+  <si>
+    <t>Volume recovered (%) = 110%</t>
+  </si>
+  <si>
+    <t>(0 / 9,741) = 0 * 100 = 0%</t>
+  </si>
+  <si>
+    <t>(110 + 0 + 0) = 110 / 3 = 36.67 %</t>
+  </si>
+  <si>
+    <t>Average Scenario Average:</t>
   </si>
 </sst>
 </file>
@@ -627,72 +669,72 @@
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C2" s="12"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" s="10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C5" s="11">
-        <f>'Kingston Normal Deletion'!E29</f>
+        <f>'Kingston Normal Deletion'!E30</f>
         <v>1</v>
       </c>
       <c r="D5" s="11">
-        <f>'Kingston Secure Erase'!E29</f>
+        <f>'Kingston Secure Erase'!E30</f>
         <v>0</v>
       </c>
       <c r="E5" s="11">
-        <f>'Kingston TRIM'!E29</f>
+        <f>'Kingston TRIM'!E30</f>
         <v>0.82</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C6" s="5">
-        <f>'PNY Normal Deletion'!E29</f>
+        <f>'PNY Normal Deletion'!E30</f>
         <v>1</v>
       </c>
       <c r="D6" s="5">
-        <f>'PNY Secure Erase'!E29</f>
-        <v>0.373</v>
+        <f>'PNY Secure Erase'!F33</f>
+        <v>0.48113333333333336</v>
       </c>
       <c r="E6" s="5">
-        <f>'PNY TRIM'!E29</f>
+        <f>'PNY TRIM'!E30</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C7" s="11">
-        <f>'Samsung Normal Deletion'!E29</f>
+        <f>'Samsung Normal Deletion'!E30</f>
         <v>1</v>
       </c>
       <c r="D7" s="11">
-        <f>'Samsung Secure Erase'!E29</f>
+        <f>'Samsung Secure Erase'!E30</f>
         <v>0.99990000000000001</v>
       </c>
       <c r="E7" s="11">
-        <f>'Samsung TRIM'!E29</f>
+        <f>'Samsung TRIM'!E30</f>
         <v>1</v>
       </c>
     </row>
@@ -706,64 +748,61 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB09AFC0-6FB1-4C77-AE3B-655B9768E87D}">
-  <dimension ref="C3:I29"/>
+  <dimension ref="B2:I30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -771,36 +810,36 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
     <row r="19" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -808,42 +847,53 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="22" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
+    <row r="21" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
     <row r="26" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="29" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="6">
+    <row r="28" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="30" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="6">
         <v>1</v>
       </c>
     </row>
@@ -854,66 +904,62 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AD9687C-3D1F-4936-99D4-5F9F4BB937FB}">
-  <dimension ref="C3:J29"/>
+  <dimension ref="B2:J30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-    </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -922,37 +968,37 @@
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
     </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
     <row r="19" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -961,42 +1007,54 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
     </row>
-    <row r="22" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
+    <row r="21" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="23" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
     <row r="26" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="29" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="6">
+    <row r="28" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="30" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1007,66 +1065,63 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3B18A72-8B9C-4863-BA86-EFB0D1DCCE85}">
-  <dimension ref="C3:J29"/>
+  <dimension ref="B2:J30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-    </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1075,37 +1130,37 @@
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
     </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
     <row r="19" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -1114,42 +1169,54 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
     </row>
-    <row r="22" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
+    <row r="21" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="23" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
     <row r="26" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="29" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="6">
+    <row r="28" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="30" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1160,66 +1227,62 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFA8DF7B-E0E7-4E7C-A3E6-057CEA155643}">
-  <dimension ref="C3:J29"/>
+  <dimension ref="B2:J30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-    </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1228,37 +1291,37 @@
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
     </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
     <row r="19" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -1267,42 +1330,54 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
     </row>
-    <row r="22" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
+    <row r="21" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="23" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
     <row r="26" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>28</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="29" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="6">
+    <row r="28" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="30" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="6">
         <v>0.82</v>
       </c>
     </row>
@@ -1313,64 +1388,61 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A4C8D61-21D0-4A69-9CF1-5147970E82D1}">
-  <dimension ref="C3:I29"/>
+  <dimension ref="B2:I30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1378,36 +1450,36 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
     <row r="19" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -1415,42 +1487,53 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="22" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
+    <row r="21" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
     <row r="26" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="29" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="6">
+    <row r="28" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="30" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1461,66 +1544,116 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50CB707C-6519-4C97-8FDF-A86D461EEC63}">
-  <dimension ref="C3:J29"/>
+  <dimension ref="B2:AD33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+      <c r="N4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="X5" s="2"/>
+    </row>
+    <row r="6" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="N6" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="X6" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="Z6" s="3"/>
+      <c r="AA6" s="3"/>
+      <c r="AB6" s="3"/>
+      <c r="AC6" s="3"/>
+      <c r="AD6" s="3"/>
+    </row>
+    <row r="7" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="O7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="Y7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z7" s="3"/>
+      <c r="AA7" s="3"/>
+    </row>
+    <row r="9" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+      <c r="N9" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="X9" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+      <c r="N11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="X11" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-    </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>29</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1528,38 +1661,90 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
-    </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+      <c r="N13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+      <c r="R13" s="3"/>
+      <c r="S13" s="3"/>
+      <c r="X13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="Z13" s="3"/>
+      <c r="AA13" s="3"/>
+      <c r="AB13" s="3"/>
+      <c r="AC13" s="3"/>
+      <c r="AD13" s="3"/>
+    </row>
+    <row r="14" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="P14" s="3"/>
+      <c r="Q14" s="3"/>
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
+      <c r="X14" s="3"/>
+      <c r="Y14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z14" s="3"/>
+      <c r="AA14" s="3"/>
+      <c r="AB14" s="3"/>
+      <c r="AC14" s="3"/>
+      <c r="AD14" s="3"/>
+    </row>
+    <row r="16" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="X16" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
-    <row r="19" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="N18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="X18" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="X19" s="1"/>
+    </row>
+    <row r="20" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>31</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -1567,44 +1752,157 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
-    </row>
-    <row r="22" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+      <c r="N20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="O20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="3"/>
+      <c r="R20" s="3"/>
+      <c r="S20" s="3"/>
+      <c r="X20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z20" s="3"/>
+      <c r="AA20" s="3"/>
+      <c r="AB20" s="3"/>
+      <c r="AC20" s="3"/>
+      <c r="AD20" s="3"/>
+    </row>
+    <row r="21" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="3"/>
+      <c r="R21" s="3"/>
+      <c r="S21" s="3"/>
+      <c r="X21" s="3"/>
+      <c r="Y21" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z21" s="3"/>
+      <c r="AA21" s="3"/>
+      <c r="AB21" s="3"/>
+      <c r="AC21" s="3"/>
+      <c r="AD21" s="3"/>
+    </row>
+    <row r="23" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="N23" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="X23" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
-    <row r="26" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="N25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="X25" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="X26" s="1"/>
+    </row>
+    <row r="27" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
-    </row>
-    <row r="29" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E29" s="7">
-        <v>0.373</v>
+      <c r="N27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3"/>
+      <c r="X27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="Y27" s="3"/>
+      <c r="Z27" s="3"/>
+      <c r="AA27" s="3"/>
+      <c r="AB27" s="3"/>
+    </row>
+    <row r="28" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="3"/>
+      <c r="X28" s="3"/>
+      <c r="Y28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z28" s="3"/>
+      <c r="AA28" s="3"/>
+      <c r="AB28" s="3"/>
+    </row>
+    <row r="30" spans="3:30" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E30" s="7">
+        <v>0.40670000000000001</v>
+      </c>
+      <c r="N30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="P30" s="6">
+        <v>0.67</v>
+      </c>
+      <c r="X30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z30" s="7">
+        <v>0.36670000000000003</v>
+      </c>
+    </row>
+    <row r="33" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C33" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F33" s="7">
+        <f>AVERAGE(E30,P30,Z30)</f>
+        <v>0.48113333333333336</v>
       </c>
     </row>
   </sheetData>
@@ -1614,64 +1912,61 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6E72CD4-50E6-490C-ADC2-A0887B6CF295}">
-  <dimension ref="C3:I29"/>
+  <dimension ref="B2:I30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1679,36 +1974,36 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
     <row r="19" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -1716,42 +2011,53 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="22" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
+    <row r="21" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
     <row r="26" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="29" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="6">
+    <row r="28" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="30" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1762,139 +2068,147 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7B579EA-5086-422A-9B22-36CD78606164}">
-  <dimension ref="C3:H29"/>
+  <dimension ref="B2:H30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-    </row>
-    <row r="6" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
-    <row r="15" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+    <row r="18" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
     <row r="19" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-    </row>
-    <row r="20" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="22" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
+    <row r="21" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+    </row>
+    <row r="23" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
     <row r="26" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="29" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="6">
+    <row r="28" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="30" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1905,64 +2219,61 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ABDB967-49F5-4F32-9DB9-86FE96453817}">
-  <dimension ref="C3:I29"/>
+  <dimension ref="B2:I30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C12" s="3" t="s">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1970,36 +2281,36 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C17" s="1" t="s">
+    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
     <row r="19" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -2007,42 +2318,53 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="22" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C22" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="24" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
+    <row r="21" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
-    </row>
     <row r="26" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>36</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="29" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="7">
+    <row r="28" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="30" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="7">
         <v>0.99990000000000001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated files and references from today
</commit_message>
<xml_diff>
--- a/Full final results.xlsx
+++ b/Full final results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\Uni\Dissertation\MScProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D1F9B3-75B0-4C56-9EEB-36C270C8ADA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74E3F4F8-F466-4899-AC35-4DA6F5188306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2085" windowWidth="29040" windowHeight="16440" xr2:uid="{A71FE66F-C5AB-4BD0-A1DF-C1EC892D38EE}"/>
+    <workbookView xWindow="38280" yWindow="2085" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="5" xr2:uid="{A71FE66F-C5AB-4BD0-A1DF-C1EC892D38EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="11" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="70">
   <si>
     <t>Volume</t>
   </si>
@@ -217,6 +217,33 @@
   </si>
   <si>
     <t>Average Scenario Average:</t>
+  </si>
+  <si>
+    <t>Sanitisation Technique</t>
+  </si>
+  <si>
+    <t>SSD 1 (Kingston)</t>
+  </si>
+  <si>
+    <t>SSD 2 (PNY)</t>
+  </si>
+  <si>
+    <t>SSD 3 (Samsung)</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>Standard Deletion</t>
+  </si>
+  <si>
+    <t>TRIM</t>
+  </si>
+  <si>
+    <t>Secure Erase</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
   </si>
 </sst>
 </file>
@@ -659,21 +686,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C25A81D0-3CBC-4521-9A86-1E03FFA15FCF}">
-  <dimension ref="B2:E7"/>
+  <dimension ref="B2:F18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
     <col min="3" max="3" width="32.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="29.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
         <v>43</v>
       </c>
       <c r="C2" s="12"/>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="10" t="s">
         <v>42</v>
       </c>
@@ -687,7 +715,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
         <v>34</v>
       </c>
@@ -704,7 +732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
         <v>35</v>
       </c>
@@ -721,7 +749,7 @@
         <v>0.48113333333333336</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
         <v>36</v>
       </c>
@@ -735,6 +763,130 @@
       </c>
       <c r="E7" s="11">
         <f>'Samsung Secure Erase'!E30</f>
+        <v>0.99990000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="11">
+        <v>1</v>
+      </c>
+      <c r="D11" s="11">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11">
+        <v>1</v>
+      </c>
+      <c r="F11" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0.82</v>
+      </c>
+      <c r="D12" s="5">
+        <v>1</v>
+      </c>
+      <c r="E12" s="5">
+        <v>1</v>
+      </c>
+      <c r="F12" s="5">
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="11">
+        <v>0</v>
+      </c>
+      <c r="D13" s="11">
+        <v>0.48110000000000003</v>
+      </c>
+      <c r="E13" s="11">
+        <v>0.99990000000000001</v>
+      </c>
+      <c r="F13" s="11">
+        <v>0.49370000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="11">
+        <v>1</v>
+      </c>
+      <c r="D16" s="11">
+        <v>0.82</v>
+      </c>
+      <c r="E16" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="5">
+        <v>1</v>
+      </c>
+      <c r="E17" s="5">
+        <v>0.48110000000000003</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="11">
+        <v>1</v>
+      </c>
+      <c r="D18" s="11">
+        <v>1</v>
+      </c>
+      <c r="E18" s="11">
         <v>0.99990000000000001</v>
       </c>
     </row>

</xml_diff>